<commit_message>
Fixing formatting for HTML generator
</commit_message>
<xml_diff>
--- a/data/oer-catalog-2024-2025.xlsx
+++ b/data/oer-catalog-2024-2025.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{27D11BC1-35FF-4E43-9830-75048CA005DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elliotgalvis/Downloads/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72EF4B2B-B60A-3C49-8D0D-3A2CB405A5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="780" windowWidth="30200" windowHeight="20640" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalog" sheetId="6" r:id="rId1"/>
@@ -1752,7 +1757,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1830,19 +1835,19 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0F374F"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2238,9 +2243,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2278,7 +2283,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2384,7 +2389,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2526,7 +2531,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2552,18 +2557,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C78B0D9-715E-4EDD-989F-8CB33D4C8A77}">
   <dimension ref="A1:L271"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" style="7" customWidth="1"/>
-    <col min="2" max="2" width="33.7109375" style="7" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="24.85546875" style="7" customWidth="1"/>
-    <col min="6" max="6" width="24.85546875" style="8" customWidth="1"/>
-    <col min="7" max="7" width="29.7109375" style="8" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="33.6640625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="21.5" style="7" customWidth="1"/>
+    <col min="4" max="4" width="19.5" style="2" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" style="8" customWidth="1"/>
+    <col min="7" max="7" width="29.6640625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="6" customFormat="1" ht="46.5" customHeight="1">
+    <row r="1" spans="1:7" s="6" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
@@ -2586,7 +2591,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="9" customFormat="1" ht="24">
+    <row r="2" spans="1:7" s="9" customFormat="1" ht="28" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>7</v>
       </c>
@@ -2609,7 +2614,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="9" customFormat="1">
+    <row r="3" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="17" t="s">
         <v>7</v>
       </c>
@@ -2632,7 +2637,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="9" customFormat="1" ht="24">
+    <row r="4" spans="1:7" s="9" customFormat="1" ht="28" x14ac:dyDescent="0.2">
       <c r="A4" s="17" t="s">
         <v>7</v>
       </c>
@@ -2655,7 +2660,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="11" customFormat="1" ht="24">
+    <row r="5" spans="1:7" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>7</v>
       </c>
@@ -2678,7 +2683,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="24">
+    <row r="6" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
         <v>7</v>
       </c>
@@ -2701,7 +2706,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="24">
+    <row r="7" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
         <v>7</v>
       </c>
@@ -2724,7 +2729,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="234" customHeight="1">
+    <row r="8" spans="1:7" ht="234" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
         <v>7</v>
       </c>
@@ -2747,7 +2752,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
         <v>38</v>
       </c>
@@ -2770,7 +2775,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="24">
+    <row r="10" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="17" t="s">
         <v>38</v>
       </c>
@@ -2793,7 +2798,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="24">
+    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.2">
       <c r="A11" s="24" t="s">
         <v>45</v>
       </c>
@@ -2816,7 +2821,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="24">
+    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.2">
       <c r="A12" s="24" t="s">
         <v>45</v>
       </c>
@@ -2839,7 +2844,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="24">
+    <row r="13" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="24" t="s">
         <v>45</v>
       </c>
@@ -2862,7 +2867,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="36">
+    <row r="14" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A14" s="24" t="s">
         <v>45</v>
       </c>
@@ -2885,7 +2890,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="24">
+    <row r="15" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A15" s="24" t="s">
         <v>45</v>
       </c>
@@ -2908,7 +2913,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="24">
+    <row r="16" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A16" s="24" t="s">
         <v>45</v>
       </c>
@@ -2931,7 +2936,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="24">
+    <row r="17" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A17" s="24" t="s">
         <v>45</v>
       </c>
@@ -2954,7 +2959,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="24">
+    <row r="18" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A18" s="24" t="s">
         <v>45</v>
       </c>
@@ -2977,7 +2982,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="24">
+    <row r="19" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A19" s="24" t="s">
         <v>45</v>
       </c>
@@ -3000,7 +3005,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="24">
+    <row r="20" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="24" t="s">
         <v>45</v>
       </c>
@@ -3023,7 +3028,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="24">
+    <row r="21" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A21" s="24" t="s">
         <v>45</v>
       </c>
@@ -3046,7 +3051,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="24">
+    <row r="22" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A22" s="24" t="s">
         <v>45</v>
       </c>
@@ -3069,7 +3074,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="36">
+    <row r="23" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A23" s="24" t="s">
         <v>45</v>
       </c>
@@ -3092,7 +3097,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="36">
+    <row r="24" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A24" s="24" t="s">
         <v>45</v>
       </c>
@@ -3115,7 +3120,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="24">
+    <row r="25" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A25" s="24" t="s">
         <v>45</v>
       </c>
@@ -3138,7 +3143,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="24">
+    <row r="26" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A26" s="24" t="s">
         <v>45</v>
       </c>
@@ -3161,7 +3166,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="24" t="s">
         <v>101</v>
       </c>
@@ -3184,7 +3189,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="24">
+    <row r="28" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A28" s="24" t="s">
         <v>101</v>
       </c>
@@ -3207,7 +3212,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="24">
+    <row r="29" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A29" s="24" t="s">
         <v>101</v>
       </c>
@@ -3230,7 +3235,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="42" customHeight="1">
+    <row r="30" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="24" t="s">
         <v>101</v>
       </c>
@@ -3253,7 +3258,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="24">
+    <row r="31" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A31" s="24" t="s">
         <v>101</v>
       </c>
@@ -3276,7 +3281,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="24">
+    <row r="32" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A32" s="24" t="s">
         <v>119</v>
       </c>
@@ -3299,7 +3304,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="24">
+    <row r="33" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A33" s="24" t="s">
         <v>119</v>
       </c>
@@ -3322,7 +3327,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:7" s="9" customFormat="1" ht="36">
+    <row r="34" spans="1:7" s="9" customFormat="1" ht="42" x14ac:dyDescent="0.2">
       <c r="A34" s="24" t="s">
         <v>119</v>
       </c>
@@ -3345,7 +3350,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="24">
+    <row r="35" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="24" t="s">
         <v>131</v>
       </c>
@@ -3368,7 +3373,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="24">
+    <row r="36" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A36" s="24" t="s">
         <v>131</v>
       </c>
@@ -3391,7 +3396,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="24">
+    <row r="37" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A37" s="24" t="s">
         <v>131</v>
       </c>
@@ -3414,7 +3419,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="24">
+    <row r="38" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A38" s="24" t="s">
         <v>131</v>
       </c>
@@ -3437,7 +3442,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="33" customHeight="1">
+    <row r="39" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="24" t="s">
         <v>131</v>
       </c>
@@ -3460,7 +3465,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="104.25" customHeight="1">
+    <row r="40" spans="1:7" ht="104.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="24" t="s">
         <v>131</v>
       </c>
@@ -3483,7 +3488,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="27" customHeight="1">
+    <row r="41" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="24" t="s">
         <v>131</v>
       </c>
@@ -3506,7 +3511,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="41.25" customHeight="1">
+    <row r="42" spans="1:7" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="24" t="s">
         <v>131</v>
       </c>
@@ -3529,7 +3534,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="24">
+    <row r="43" spans="1:7" ht="29" x14ac:dyDescent="0.2">
       <c r="A43" s="24" t="s">
         <v>131</v>
       </c>
@@ -3552,7 +3557,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="24">
+    <row r="44" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A44" s="24" t="s">
         <v>131</v>
       </c>
@@ -3575,7 +3580,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="41.25" customHeight="1">
+    <row r="45" spans="1:7" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="24" t="s">
         <v>131</v>
       </c>
@@ -3598,7 +3603,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="28.5" customHeight="1">
+    <row r="46" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="24" t="s">
         <v>131</v>
       </c>
@@ -3621,7 +3626,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="24" t="s">
         <v>131</v>
       </c>
@@ -3644,7 +3649,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="24">
+    <row r="48" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A48" s="24" t="s">
         <v>175</v>
       </c>
@@ -3667,7 +3672,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="24">
+    <row r="49" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A49" s="24" t="s">
         <v>175</v>
       </c>
@@ -3690,7 +3695,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="50" spans="1:7" s="9" customFormat="1" ht="36">
+    <row r="50" spans="1:7" s="9" customFormat="1" ht="42" x14ac:dyDescent="0.2">
       <c r="A50" s="17" t="s">
         <v>175</v>
       </c>
@@ -3713,7 +3718,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="24">
+    <row r="51" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A51" s="24" t="s">
         <v>175</v>
       </c>
@@ -3736,7 +3741,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="24">
+    <row r="52" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A52" s="24" t="s">
         <v>175</v>
       </c>
@@ -3759,7 +3764,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="53" spans="1:7" s="9" customFormat="1" ht="36">
+    <row r="53" spans="1:7" s="9" customFormat="1" ht="42" x14ac:dyDescent="0.2">
       <c r="A53" s="17" t="s">
         <v>175</v>
       </c>
@@ -3782,7 +3787,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="41.25" customHeight="1">
+    <row r="54" spans="1:7" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="24" t="s">
         <v>175</v>
       </c>
@@ -3805,7 +3810,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="24">
+    <row r="55" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A55" s="24" t="s">
         <v>175</v>
       </c>
@@ -3828,7 +3833,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="36">
+    <row r="56" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A56" s="24" t="s">
         <v>175</v>
       </c>
@@ -3851,7 +3856,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="53.25" customHeight="1">
+    <row r="57" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="24" t="s">
         <v>175</v>
       </c>
@@ -3874,7 +3879,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="72">
+    <row r="58" spans="1:7" ht="84" x14ac:dyDescent="0.2">
       <c r="A58" s="24" t="s">
         <v>175</v>
       </c>
@@ -3897,7 +3902,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="31.5" customHeight="1">
+    <row r="59" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="24" t="s">
         <v>175</v>
       </c>
@@ -3920,7 +3925,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="24">
+    <row r="60" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A60" s="24" t="s">
         <v>213</v>
       </c>
@@ -3943,7 +3948,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="24">
+    <row r="61" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A61" s="24" t="s">
         <v>213</v>
       </c>
@@ -3966,7 +3971,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="24">
+    <row r="62" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A62" s="24" t="s">
         <v>213</v>
       </c>
@@ -3989,7 +3994,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="24">
+    <row r="63" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A63" s="24" t="s">
         <v>213</v>
       </c>
@@ -4012,7 +4017,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="24">
+    <row r="64" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A64" s="24" t="s">
         <v>213</v>
       </c>
@@ -4035,7 +4040,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="65" spans="1:7">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" s="24" t="s">
         <v>213</v>
       </c>
@@ -4058,7 +4063,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="66" spans="1:7">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" s="24" t="s">
         <v>213</v>
       </c>
@@ -4081,7 +4086,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="42.75" customHeight="1">
+    <row r="67" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="24" t="s">
         <v>213</v>
       </c>
@@ -4104,7 +4109,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="24">
+    <row r="68" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A68" s="24" t="s">
         <v>213</v>
       </c>
@@ -4127,7 +4132,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="29.25" customHeight="1">
+    <row r="69" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="24" t="s">
         <v>213</v>
       </c>
@@ -4150,7 +4155,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="24">
+    <row r="70" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A70" s="24" t="s">
         <v>213</v>
       </c>
@@ -4173,7 +4178,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="24">
+    <row r="71" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A71" s="24" t="s">
         <v>213</v>
       </c>
@@ -4196,7 +4201,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="24">
+    <row r="72" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A72" s="24" t="s">
         <v>213</v>
       </c>
@@ -4219,7 +4224,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="73" spans="1:7" ht="24">
+    <row r="73" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A73" s="24" t="s">
         <v>213</v>
       </c>
@@ -4242,7 +4247,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="24">
+    <row r="74" spans="1:7" ht="29" x14ac:dyDescent="0.2">
       <c r="A74" s="24" t="s">
         <v>213</v>
       </c>
@@ -4265,7 +4270,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="24">
+    <row r="75" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A75" s="24" t="s">
         <v>213</v>
       </c>
@@ -4288,7 +4293,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="24">
+    <row r="76" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A76" s="24" t="s">
         <v>213</v>
       </c>
@@ -4311,7 +4316,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="77" spans="1:7" s="9" customFormat="1" ht="24">
+    <row r="77" spans="1:7" s="9" customFormat="1" ht="28" x14ac:dyDescent="0.2">
       <c r="A77" s="17" t="s">
         <v>213</v>
       </c>
@@ -4334,7 +4339,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="78" spans="1:7" ht="24">
+    <row r="78" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A78" s="24" t="s">
         <v>213</v>
       </c>
@@ -4357,7 +4362,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="24">
+    <row r="79" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A79" s="24" t="s">
         <v>213</v>
       </c>
@@ -4380,7 +4385,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="80" spans="1:7">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" s="24" t="s">
         <v>213</v>
       </c>
@@ -4403,7 +4408,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" s="24" t="s">
         <v>213</v>
       </c>
@@ -4426,7 +4431,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="82" spans="1:7" ht="24">
+    <row r="82" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A82" s="24" t="s">
         <v>213</v>
       </c>
@@ -4449,7 +4454,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="83" spans="1:7" ht="24">
+    <row r="83" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A83" s="24" t="s">
         <v>213</v>
       </c>
@@ -4472,7 +4477,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="84" spans="1:7" ht="36">
+    <row r="84" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A84" s="24" t="s">
         <v>213</v>
       </c>
@@ -4495,7 +4500,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="36">
+    <row r="85" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A85" s="24" t="s">
         <v>213</v>
       </c>
@@ -4518,7 +4523,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="86" spans="1:7" ht="24">
+    <row r="86" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A86" s="24" t="s">
         <v>213</v>
       </c>
@@ -4541,7 +4546,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="87" spans="1:7" ht="24">
+    <row r="87" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A87" s="24" t="s">
         <v>213</v>
       </c>
@@ -4564,7 +4569,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="88" spans="1:7" ht="24">
+    <row r="88" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A88" s="17" t="s">
         <v>38</v>
       </c>
@@ -4587,7 +4592,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="89" spans="1:7" ht="24">
+    <row r="89" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A89" s="17" t="s">
         <v>38</v>
       </c>
@@ -4610,7 +4615,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="90" spans="1:7" ht="24">
+    <row r="90" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A90" s="17" t="s">
         <v>38</v>
       </c>
@@ -4633,7 +4638,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="91" spans="1:7" ht="33" customHeight="1">
+    <row r="91" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="17" t="s">
         <v>38</v>
       </c>
@@ -4656,7 +4661,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="28.5" customHeight="1">
+    <row r="92" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="17" t="s">
         <v>38</v>
       </c>
@@ -4679,7 +4684,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="24">
+    <row r="93" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A93" s="17" t="s">
         <v>38</v>
       </c>
@@ -4702,7 +4707,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="24">
+    <row r="94" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A94" s="17" t="s">
         <v>38</v>
       </c>
@@ -4725,7 +4730,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="48">
+    <row r="95" spans="1:7" ht="56" x14ac:dyDescent="0.2">
       <c r="A95" s="17" t="s">
         <v>38</v>
       </c>
@@ -4748,7 +4753,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="24">
+    <row r="96" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A96" s="17" t="s">
         <v>38</v>
       </c>
@@ -4771,7 +4776,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="24">
+    <row r="97" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A97" s="17" t="s">
         <v>38</v>
       </c>
@@ -4794,7 +4799,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="98" spans="1:7" s="11" customFormat="1" ht="36" hidden="1">
+    <row r="98" spans="1:7" s="11" customFormat="1" ht="42" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" s="17" t="s">
         <v>38</v>
       </c>
@@ -4817,7 +4822,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="41.25" customHeight="1">
+    <row r="99" spans="1:7" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="17" t="s">
         <v>38</v>
       </c>
@@ -4840,7 +4845,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="42" customHeight="1">
+    <row r="100" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="17" t="s">
         <v>38</v>
       </c>
@@ -4863,7 +4868,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="24">
+    <row r="101" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A101" s="24" t="s">
         <v>335</v>
       </c>
@@ -4886,7 +4891,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="102" spans="1:7">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" s="24" t="s">
         <v>340</v>
       </c>
@@ -4909,7 +4914,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="103" spans="1:7">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" s="24" t="s">
         <v>340</v>
       </c>
@@ -4932,7 +4937,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="24">
+    <row r="104" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A104" s="24" t="s">
         <v>340</v>
       </c>
@@ -4955,7 +4960,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="48">
+    <row r="105" spans="1:7" ht="56" x14ac:dyDescent="0.2">
       <c r="A105" s="24" t="s">
         <v>340</v>
       </c>
@@ -4978,7 +4983,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="106" spans="1:7" ht="36">
+    <row r="106" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A106" s="24" t="s">
         <v>353</v>
       </c>
@@ -5001,7 +5006,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="24">
+    <row r="107" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A107" s="24" t="s">
         <v>353</v>
       </c>
@@ -5024,7 +5029,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="24">
+    <row r="108" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A108" s="24" t="s">
         <v>353</v>
       </c>
@@ -5047,7 +5052,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="48">
+    <row r="109" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A109" s="24" t="s">
         <v>353</v>
       </c>
@@ -5070,7 +5075,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="24">
+    <row r="110" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A110" s="24" t="s">
         <v>353</v>
       </c>
@@ -5093,7 +5098,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="24">
+    <row r="111" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A111" s="24" t="s">
         <v>353</v>
       </c>
@@ -5116,7 +5121,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="108.75" customHeight="1">
+    <row r="112" spans="1:7" ht="108.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="24" t="s">
         <v>353</v>
       </c>
@@ -5139,7 +5144,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="113" spans="1:7" ht="83.25" customHeight="1">
+    <row r="113" spans="1:7" ht="83.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="24" t="s">
         <v>375</v>
       </c>
@@ -5162,7 +5167,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="114" spans="1:7" ht="24">
+    <row r="114" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A114" s="24" t="s">
         <v>375</v>
       </c>
@@ -5185,7 +5190,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="115" spans="1:7" ht="24">
+    <row r="115" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A115" s="24" t="s">
         <v>375</v>
       </c>
@@ -5208,7 +5213,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="34.5" customHeight="1">
+    <row r="116" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="24" t="s">
         <v>375</v>
       </c>
@@ -5231,7 +5236,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="24">
+    <row r="117" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A117" s="24" t="s">
         <v>375</v>
       </c>
@@ -5254,7 +5259,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="24">
+    <row r="118" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A118" s="24" t="s">
         <v>375</v>
       </c>
@@ -5277,7 +5282,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="24">
+    <row r="119" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A119" s="24" t="s">
         <v>375</v>
       </c>
@@ -5300,7 +5305,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="120" spans="1:7" ht="24">
+    <row r="120" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A120" s="24" t="s">
         <v>375</v>
       </c>
@@ -5323,7 +5328,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="121" spans="1:7" s="10" customFormat="1" ht="36">
+    <row r="121" spans="1:7" s="10" customFormat="1" ht="43" x14ac:dyDescent="0.2">
       <c r="A121" s="17" t="s">
         <v>375</v>
       </c>
@@ -5346,7 +5351,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="122" spans="1:7" s="10" customFormat="1" ht="36">
+    <row r="122" spans="1:7" s="10" customFormat="1" ht="43" x14ac:dyDescent="0.2">
       <c r="A122" s="17" t="s">
         <v>375</v>
       </c>
@@ -5369,7 +5374,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="123" spans="1:7" ht="24">
+    <row r="123" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A123" s="24" t="s">
         <v>375</v>
       </c>
@@ -5392,7 +5397,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="124" spans="1:7" ht="24">
+    <row r="124" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A124" s="24" t="s">
         <v>375</v>
       </c>
@@ -5415,7 +5420,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="125" spans="1:7" ht="24">
+    <row r="125" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A125" s="24" t="s">
         <v>375</v>
       </c>
@@ -5438,7 +5443,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="126" spans="1:7" ht="24">
+    <row r="126" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A126" s="24" t="s">
         <v>375</v>
       </c>
@@ -5461,7 +5466,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="127" spans="1:7" ht="24">
+    <row r="127" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A127" s="24" t="s">
         <v>375</v>
       </c>
@@ -5484,7 +5489,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="24">
+    <row r="128" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A128" s="24" t="s">
         <v>375</v>
       </c>
@@ -5507,7 +5512,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="24">
+    <row r="129" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A129" s="24" t="s">
         <v>375</v>
       </c>
@@ -5530,7 +5535,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="24">
+    <row r="130" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A130" s="24" t="s">
         <v>375</v>
       </c>
@@ -5553,7 +5558,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="24">
+    <row r="131" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A131" s="24" t="s">
         <v>428</v>
       </c>
@@ -5576,7 +5581,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="132" spans="1:7">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A132" s="24" t="s">
         <v>428</v>
       </c>
@@ -5599,7 +5604,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="133" spans="1:7">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A133" s="24" t="s">
         <v>428</v>
       </c>
@@ -5622,7 +5627,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="48">
+    <row r="134" spans="1:7" ht="56" x14ac:dyDescent="0.2">
       <c r="A134" s="24" t="s">
         <v>428</v>
       </c>
@@ -5645,7 +5650,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="24">
+    <row r="135" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A135" s="24" t="s">
         <v>428</v>
       </c>
@@ -5668,7 +5673,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="24">
+    <row r="136" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A136" s="24" t="s">
         <v>428</v>
       </c>
@@ -5691,7 +5696,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="61.5" customHeight="1">
+    <row r="137" spans="1:7" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="24" t="s">
         <v>447</v>
       </c>
@@ -5714,7 +5719,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="36">
+    <row r="138" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A138" s="24" t="s">
         <v>447</v>
       </c>
@@ -5737,7 +5742,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="24">
+    <row r="139" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A139" s="24" t="s">
         <v>447</v>
       </c>
@@ -5760,7 +5765,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="24">
+    <row r="140" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A140" s="24" t="s">
         <v>447</v>
       </c>
@@ -5783,7 +5788,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="24">
+    <row r="141" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A141" s="24" t="s">
         <v>447</v>
       </c>
@@ -5806,7 +5811,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="24">
+    <row r="142" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A142" s="24" t="s">
         <v>447</v>
       </c>
@@ -5829,7 +5834,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="24">
+    <row r="143" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A143" s="24" t="s">
         <v>447</v>
       </c>
@@ -5852,7 +5857,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="24">
+    <row r="144" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A144" s="24" t="s">
         <v>447</v>
       </c>
@@ -5875,7 +5880,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="145" spans="1:12" ht="24">
+    <row r="145" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A145" s="24" t="s">
         <v>447</v>
       </c>
@@ -5898,7 +5903,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="146" spans="1:12" ht="24">
+    <row r="146" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A146" s="24" t="s">
         <v>447</v>
       </c>
@@ -5921,7 +5926,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="147" spans="1:12" ht="24">
+    <row r="147" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A147" s="24" t="s">
         <v>447</v>
       </c>
@@ -5944,7 +5949,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="148" spans="1:12" ht="24">
+    <row r="148" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A148" s="24" t="s">
         <v>447</v>
       </c>
@@ -5967,7 +5972,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="149" spans="1:12" ht="24">
+    <row r="149" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A149" s="24" t="s">
         <v>447</v>
       </c>
@@ -5990,7 +5995,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="150" spans="1:12" ht="24">
+    <row r="150" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A150" s="24" t="s">
         <v>447</v>
       </c>
@@ -6013,7 +6018,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="151" spans="1:12" ht="24">
+    <row r="151" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A151" s="24" t="s">
         <v>447</v>
       </c>
@@ -6036,7 +6041,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="152" spans="1:12">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A152" s="24" t="s">
         <v>447</v>
       </c>
@@ -6059,7 +6064,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="153" spans="1:12" ht="39" customHeight="1">
+    <row r="153" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="24" t="s">
         <v>483</v>
       </c>
@@ -6082,7 +6087,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="154" spans="1:12" s="12" customFormat="1" ht="24">
+    <row r="154" spans="1:12" s="12" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A154" s="63" t="s">
         <v>131</v>
       </c>
@@ -6105,7 +6110,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="155" spans="1:12">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A155" s="64" t="s">
         <v>483</v>
       </c>
@@ -6128,7 +6133,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="156" spans="1:12" ht="30.75">
+    <row r="156" spans="1:12" ht="280" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>483</v>
       </c>
@@ -6164,7 +6169,7 @@
       </c>
       <c r="L156" s="46"/>
     </row>
-    <row r="157" spans="1:12" ht="30.75">
+    <row r="157" spans="1:12" ht="280" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>483</v>
       </c>
@@ -6200,7 +6205,7 @@
       </c>
       <c r="L157" s="49"/>
     </row>
-    <row r="158" spans="1:12" ht="30.75">
+    <row r="158" spans="1:12" ht="280" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>483</v>
       </c>
@@ -6236,7 +6241,7 @@
       </c>
       <c r="L158" s="49"/>
     </row>
-    <row r="159" spans="1:12" ht="30.75">
+    <row r="159" spans="1:12" ht="280" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>483</v>
       </c>
@@ -6272,7 +6277,7 @@
       </c>
       <c r="L159" s="50"/>
     </row>
-    <row r="160" spans="1:12" ht="29.25">
+    <row r="160" spans="1:12" ht="280" x14ac:dyDescent="0.2">
       <c r="A160" s="69" t="s">
         <v>483</v>
       </c>
@@ -6308,7 +6313,7 @@
       </c>
       <c r="L160" s="53"/>
     </row>
-    <row r="161" spans="1:12" ht="29.25">
+    <row r="161" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A161" s="69" t="s">
         <v>483</v>
       </c>
@@ -6344,7 +6349,7 @@
       </c>
       <c r="L161" s="53"/>
     </row>
-    <row r="162" spans="1:12">
+    <row r="162" spans="1:12" ht="288" x14ac:dyDescent="0.2">
       <c r="A162" s="69" t="s">
         <v>483</v>
       </c>
@@ -6380,7 +6385,7 @@
       </c>
       <c r="L162" s="58"/>
     </row>
-    <row r="163" spans="1:12" ht="29.25">
+    <row r="163" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A163" s="69" t="s">
         <v>483</v>
       </c>
@@ -6416,7 +6421,7 @@
       </c>
       <c r="L163" s="58"/>
     </row>
-    <row r="164" spans="1:12" ht="24">
+    <row r="164" spans="1:12" ht="320" x14ac:dyDescent="0.2">
       <c r="A164" s="69" t="s">
         <v>483</v>
       </c>
@@ -6452,276 +6457,276 @@
       </c>
       <c r="L164" s="58"/>
     </row>
-    <row r="165" spans="1:12">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A165" s="8"/>
       <c r="B165" s="8"/>
       <c r="C165" s="8"/>
       <c r="D165" s="8"/>
       <c r="E165" s="8"/>
     </row>
-    <row r="166" spans="1:12">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A166" s="8"/>
       <c r="B166" s="8"/>
       <c r="C166" s="8"/>
       <c r="D166" s="8"/>
       <c r="E166" s="8"/>
     </row>
-    <row r="167" spans="1:12">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A167" s="8"/>
       <c r="B167" s="8"/>
       <c r="C167" s="8"/>
       <c r="D167" s="8"/>
       <c r="E167" s="8"/>
     </row>
-    <row r="168" spans="1:12">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A168" s="8"/>
       <c r="B168" s="8"/>
       <c r="C168" s="8"/>
       <c r="D168" s="8"/>
       <c r="E168" s="8"/>
     </row>
-    <row r="169" spans="1:12">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A169" s="8"/>
       <c r="B169" s="8"/>
       <c r="C169" s="8"/>
       <c r="D169" s="8"/>
       <c r="E169" s="8"/>
     </row>
-    <row r="170" spans="1:12">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A170" s="8"/>
       <c r="B170" s="8"/>
       <c r="C170" s="8"/>
       <c r="D170" s="8"/>
       <c r="E170" s="8"/>
     </row>
-    <row r="171" spans="1:12">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A171" s="8"/>
       <c r="B171" s="8"/>
       <c r="C171" s="8"/>
       <c r="D171" s="8"/>
       <c r="E171" s="8"/>
     </row>
-    <row r="172" spans="1:12">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A172" s="8"/>
       <c r="B172" s="8"/>
       <c r="C172" s="8"/>
       <c r="D172" s="8"/>
       <c r="E172" s="8"/>
     </row>
-    <row r="173" spans="1:12">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A173" s="8"/>
       <c r="B173" s="8"/>
       <c r="C173" s="8"/>
       <c r="D173" s="8"/>
       <c r="E173" s="8"/>
     </row>
-    <row r="174" spans="1:12">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A174" s="8"/>
       <c r="B174" s="8"/>
       <c r="C174" s="8"/>
       <c r="D174" s="8"/>
       <c r="E174" s="8"/>
     </row>
-    <row r="175" spans="1:12">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A175" s="8"/>
       <c r="B175" s="8"/>
       <c r="C175" s="8"/>
       <c r="D175" s="8"/>
       <c r="E175" s="8"/>
     </row>
-    <row r="176" spans="1:12">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A176" s="8"/>
       <c r="B176" s="8"/>
       <c r="C176" s="8"/>
       <c r="D176" s="8"/>
       <c r="E176" s="8"/>
     </row>
-    <row r="177" spans="1:5">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177" s="8"/>
       <c r="B177" s="8"/>
       <c r="C177" s="8"/>
       <c r="D177" s="8"/>
       <c r="E177" s="8"/>
     </row>
-    <row r="178" spans="1:5">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178" s="8"/>
       <c r="B178" s="8"/>
       <c r="C178" s="8"/>
       <c r="D178" s="8"/>
       <c r="E178" s="8"/>
     </row>
-    <row r="179" spans="1:5">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A179" s="8"/>
       <c r="B179" s="8"/>
       <c r="C179" s="8"/>
       <c r="D179" s="8"/>
       <c r="E179" s="8"/>
     </row>
-    <row r="180" spans="1:5">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A180" s="8"/>
       <c r="B180" s="8"/>
       <c r="C180" s="8"/>
       <c r="D180" s="8"/>
       <c r="E180" s="8"/>
     </row>
-    <row r="181" spans="1:5">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A181" s="8"/>
       <c r="B181" s="8"/>
       <c r="C181" s="8"/>
       <c r="D181" s="8"/>
       <c r="E181" s="8"/>
     </row>
-    <row r="182" spans="1:5">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A182" s="8"/>
       <c r="B182" s="8"/>
       <c r="C182" s="8"/>
       <c r="D182" s="8"/>
       <c r="E182" s="8"/>
     </row>
-    <row r="183" spans="1:5">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A183" s="8"/>
       <c r="B183" s="8"/>
       <c r="C183" s="8"/>
       <c r="D183" s="8"/>
       <c r="E183" s="8"/>
     </row>
-    <row r="184" spans="1:5">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A184" s="8"/>
       <c r="B184" s="8"/>
       <c r="C184" s="8"/>
       <c r="D184" s="8"/>
       <c r="E184" s="8"/>
     </row>
-    <row r="185" spans="1:5">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A185" s="8"/>
       <c r="B185" s="8"/>
       <c r="C185" s="8"/>
       <c r="D185" s="8"/>
       <c r="E185" s="8"/>
     </row>
-    <row r="186" spans="1:5">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A186" s="8"/>
       <c r="B186" s="8"/>
       <c r="C186" s="8"/>
       <c r="D186" s="8"/>
       <c r="E186" s="8"/>
     </row>
-    <row r="187" spans="1:5">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187" s="8"/>
       <c r="B187" s="8"/>
       <c r="C187" s="8"/>
       <c r="D187" s="8"/>
       <c r="E187" s="8"/>
     </row>
-    <row r="188" spans="1:5">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A188" s="8"/>
       <c r="B188" s="8"/>
       <c r="C188" s="8"/>
       <c r="D188" s="8"/>
       <c r="E188" s="8"/>
     </row>
-    <row r="189" spans="1:5">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A189" s="8"/>
       <c r="B189" s="8"/>
       <c r="C189" s="8"/>
       <c r="D189" s="8"/>
       <c r="E189" s="8"/>
     </row>
-    <row r="190" spans="1:5">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A190" s="8"/>
       <c r="B190" s="8"/>
       <c r="C190" s="8"/>
       <c r="D190" s="8"/>
       <c r="E190" s="8"/>
     </row>
-    <row r="191" spans="1:5">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A191" s="8"/>
       <c r="B191" s="8"/>
       <c r="C191" s="8"/>
       <c r="D191" s="8"/>
       <c r="E191" s="8"/>
     </row>
-    <row r="192" spans="1:5">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A192" s="8"/>
       <c r="B192" s="8"/>
       <c r="C192" s="8"/>
       <c r="D192" s="8"/>
       <c r="E192" s="8"/>
     </row>
-    <row r="193" spans="1:5">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A193" s="8"/>
       <c r="B193" s="8"/>
       <c r="C193" s="8"/>
       <c r="D193" s="8"/>
       <c r="E193" s="8"/>
     </row>
-    <row r="194" spans="1:5">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194" s="8"/>
       <c r="B194" s="8"/>
       <c r="C194" s="8"/>
       <c r="D194" s="8"/>
       <c r="E194" s="8"/>
     </row>
-    <row r="195" spans="1:5">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195" s="8"/>
       <c r="B195" s="8"/>
       <c r="C195" s="8"/>
       <c r="D195" s="8"/>
       <c r="E195" s="8"/>
     </row>
-    <row r="196" spans="1:5">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196" s="8"/>
       <c r="B196" s="8"/>
       <c r="C196" s="8"/>
       <c r="D196" s="8"/>
       <c r="E196" s="8"/>
     </row>
-    <row r="197" spans="1:5">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197" s="8"/>
       <c r="B197" s="8"/>
       <c r="C197" s="8"/>
       <c r="D197" s="8"/>
       <c r="E197" s="8"/>
     </row>
-    <row r="198" spans="1:5">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198" s="8"/>
       <c r="B198" s="8"/>
       <c r="C198" s="8"/>
       <c r="D198" s="8"/>
       <c r="E198" s="8"/>
     </row>
-    <row r="199" spans="1:5">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A199" s="8"/>
       <c r="B199" s="8"/>
       <c r="C199" s="8"/>
       <c r="D199" s="8"/>
       <c r="E199" s="8"/>
     </row>
-    <row r="200" spans="1:5">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A200" s="8"/>
       <c r="B200" s="8"/>
       <c r="C200" s="8"/>
       <c r="D200" s="8"/>
       <c r="E200" s="8"/>
     </row>
-    <row r="201" spans="1:5">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A201" s="8"/>
       <c r="B201" s="8"/>
       <c r="C201" s="8"/>
       <c r="D201" s="8"/>
       <c r="E201" s="8"/>
     </row>
-    <row r="202" spans="1:5">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A202" s="8"/>
       <c r="B202" s="8"/>
       <c r="C202" s="8"/>
       <c r="D202" s="8"/>
       <c r="E202" s="8"/>
     </row>
-    <row r="269" spans="5:5">
+    <row r="269" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E269" s="13"/>
     </row>
-    <row r="271" spans="5:5">
+    <row r="271" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E271" s="14"/>
     </row>
   </sheetData>
@@ -6908,39 +6913,39 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD006C89-1AA2-4301-A3E8-1AF42E12C555}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" style="40" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="8.5" style="40" customWidth="1"/>
+    <col min="3" max="3" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="19" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.5" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="17" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30.75">
+    <row r="1" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="42" t="s">
         <v>525</v>
       </c>
@@ -6948,7 +6953,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>45</v>
       </c>
@@ -6956,7 +6961,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>340</v>
       </c>
@@ -6964,7 +6969,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>335</v>
       </c>
@@ -6972,7 +6977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>483</v>
       </c>
@@ -6981,7 +6986,7 @@
       </c>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>101</v>
       </c>
@@ -6990,7 +6995,7 @@
       </c>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
@@ -6999,7 +7004,7 @@
       </c>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>353</v>
       </c>
@@ -7008,7 +7013,7 @@
       </c>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>375</v>
       </c>
@@ -7017,7 +7022,7 @@
       </c>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>527</v>
       </c>
@@ -7026,7 +7031,7 @@
       </c>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>131</v>
       </c>
@@ -7035,7 +7040,7 @@
       </c>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>428</v>
       </c>
@@ -7044,7 +7049,7 @@
       </c>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>528</v>
       </c>
@@ -7053,7 +7058,7 @@
       </c>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>447</v>
       </c>
@@ -7062,7 +7067,7 @@
       </c>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>213</v>
       </c>
@@ -7071,7 +7076,7 @@
       </c>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>529</v>
       </c>
@@ -7080,7 +7085,7 @@
       </c>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>530</v>
       </c>
@@ -7115,13 +7120,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F3854A-26D2-4B73-8883-41115D3B5C7C}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" customWidth="1"/>
+    <col min="1" max="1" width="30.5" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="30.75">
+    <row r="1" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>531</v>
       </c>
@@ -7129,7 +7134,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>47</v>
       </c>
@@ -7137,7 +7142,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
@@ -7145,7 +7150,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>110</v>
       </c>
@@ -7153,7 +7158,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>133</v>
       </c>
@@ -7161,7 +7166,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
@@ -7169,7 +7174,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>61</v>
       </c>
@@ -7177,7 +7182,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>167</v>
       </c>
@@ -7185,7 +7190,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>275</v>
       </c>
@@ -7193,7 +7198,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>142</v>
       </c>
@@ -7201,7 +7206,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>337</v>
       </c>
@@ -7209,7 +7214,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>103</v>
       </c>
@@ -7217,7 +7222,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>35</v>
       </c>
@@ -7225,7 +7230,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>51</v>
       </c>
@@ -7233,7 +7238,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>23</v>
       </c>
@@ -7241,7 +7246,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>15</v>
       </c>
@@ -7249,7 +7254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>28</v>
       </c>
@@ -7257,7 +7262,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>530</v>
       </c>
@@ -7292,13 +7297,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A20EE7BF-088B-4DBC-8B00-B4629CB74C85}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" style="40" customWidth="1"/>
-    <col min="2" max="2" width="8.28515625" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" style="40" customWidth="1"/>
+    <col min="2" max="2" width="8.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="30.75">
+    <row r="1" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="44" t="s">
         <v>532</v>
       </c>
@@ -7306,7 +7311,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="30.75">
+    <row r="2" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="40" t="s">
         <v>75</v>
       </c>
@@ -7314,7 +7319,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="30.75">
+    <row r="3" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="40" t="s">
         <v>68</v>
       </c>
@@ -7322,7 +7327,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1">
+    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="40" t="s">
         <v>193</v>
       </c>
@@ -7330,7 +7335,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="30.75">
+    <row r="5" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="40" t="s">
         <v>27</v>
       </c>
@@ -7338,7 +7343,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30.75">
+    <row r="6" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="40" t="s">
         <v>9</v>
       </c>
@@ -7346,7 +7351,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30.75">
+    <row r="7" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="40" t="s">
         <v>94</v>
       </c>
@@ -7354,7 +7359,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="40" t="s">
         <v>137</v>
       </c>
@@ -7362,7 +7367,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="40" t="s">
         <v>121</v>
       </c>
@@ -7370,7 +7375,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="41" t="s">
         <v>530</v>
       </c>
@@ -7385,6 +7390,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="e1fe8cf4-797e-455f-bdfc-84f59ecaf273" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ddf82700-9bfb-4fea-878c-7eefdbc7745a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A70658DA2082244F88130573F11D6B61" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="858aee249293fa9096085e62b28b992c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ddf82700-9bfb-4fea-878c-7eefdbc7745a" xmlns:ns3="e1fe8cf4-797e-455f-bdfc-84f59ecaf273" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0bb51cc068e630e42264d9068ea4c7f6" ns2:_="" ns3:_="">
     <xsd:import namespace="ddf82700-9bfb-4fea-878c-7eefdbc7745a"/>
@@ -7585,17 +7601,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="e1fe8cf4-797e-455f-bdfc-84f59ecaf273" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ddf82700-9bfb-4fea-878c-7eefdbc7745a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -7606,13 +7611,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63105CD5-8CA5-4DAD-B85E-7A49F4224C26}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB11F60C-BEA5-4032-9DEF-D983207E1747}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e1fe8cf4-797e-455f-bdfc-84f59ecaf273"/>
+    <ds:schemaRef ds:uri="ddf82700-9bfb-4fea-878c-7eefdbc7745a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB11F60C-BEA5-4032-9DEF-D983207E1747}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63105CD5-8CA5-4DAD-B85E-7A49F4224C26}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ddf82700-9bfb-4fea-878c-7eefdbc7745a"/>
+    <ds:schemaRef ds:uri="e1fe8cf4-797e-455f-bdfc-84f59ecaf273"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C1BDF07-269F-4A8A-929B-119FFB2E0C7C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C1BDF07-269F-4A8A-929B-119FFB2E0C7C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>